<commit_message>
refactor: rebrand from SwiftTranslator to PixelsSuite
- Rename project root to pixelssuite-playwright
- Update all URL references from swifttranslator.com to pixelssuite.com/chat-translator
- Fix column auto-detection bug (exact match for explicit --input-col names)
- Rewrite README with full CLI reference, setup guide (Python 3.12 venv), and result status docs
- Update .gitignore to exclude .venv and __pycache__
- Update Excel test case workbook (actual output + status columns)
</commit_message>
<xml_diff>
--- a/test_automation/Assignment 1 - Test cases.xlsx
+++ b/test_automation/Assignment 1 - Test cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Table" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -65,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -77,12 +77,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -359,22 +353,22 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I51"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="0"/>
   <cols>
     <col width="9.130000000000001" customWidth="1" style="6" min="1" max="1"/>
     <col width="12.13" customWidth="1" style="6" min="2" max="2"/>
-    <col width="43.75" customWidth="1" style="6" min="3" max="3"/>
-    <col width="41.63" customWidth="1" style="6" min="4" max="4"/>
+    <col width="332.5" customWidth="1" style="6" min="3" max="3"/>
+    <col width="281.13" customWidth="1" style="6" min="4" max="4"/>
     <col width="9.880000000000001" customWidth="1" style="6" min="5" max="5"/>
     <col width="5" customWidth="1" style="6" min="6" max="6"/>
     <col width="33" customWidth="1" style="6" min="7" max="7"/>
-    <col width="74.38" customWidth="1" style="6" min="8" max="8"/>
+    <col width="104.38" customWidth="1" style="6" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Test Case ID</t>
+          <t>TC ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -435,20 +429,24 @@
           <t>එහෙනම් අද අපි මොකක්ද කරන්නේ කියලා හිතුවේ ඔයා?</t>
         </is>
       </c>
-      <c r="E2" s="0" t="n"/>
-      <c r="F2" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>එහෙනම් අද අපි මොකද කරන්නේ කියලා හිතුවේ ඔයා?</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>Question forms</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
-        <is>
-          <t>Rationale: The sentence ends with "oya?" — a direct question asking someone what they planned to do today, matching the question-form input type.</t>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: The sentence is asking a direct question about what to do today.</t>
         </is>
       </c>
     </row>
@@ -473,19 +471,24 @@
           <t>ඒගොල්ලෝ ගියාද එතකොට?</t>
         </is>
       </c>
-      <c r="F3" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ඒ ගොල්ලෝ ගියාද එතකොට?</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Question forms</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "giyada" — the "-da" suffix is the standard Singlish interrogative marker, forming a yes/no question.</t>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: The sentence structure ends with 'da', indicating an interrogative phrase.</t>
         </is>
       </c>
     </row>
@@ -510,20 +513,24 @@
           <t>ඔය වැඩේ මේ දැන්ම ඉවර කරලා දාන්න මචන්.</t>
         </is>
       </c>
-      <c r="E4" s="0" t="n"/>
-      <c r="F4" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ඔය වැඩේ මේ දැන්ම ඉවර කරලා දාන්න මචං.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Command forms</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>Rationale: "iwara karala danna" is a direct imperative instruction telling someone to finish the task immediately, matching the command-form input type.</t>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: It is a direct instruction to finish a task immediately.</t>
         </is>
       </c>
     </row>
@@ -548,19 +555,24 @@
           <t>ගිහින් එන්න ඉස්සෙල්ලා බලන්න.</t>
         </is>
       </c>
-      <c r="F5" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ගිහින් එන්න ඉසැල්ල බලන්න.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Command forms</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>Rationale: "ghin enna isella blanna" is a sequential command — go, come back, then look — structured as a direct instruction.</t>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: It is a command instructing someone to look before leaving.</t>
         </is>
       </c>
     </row>
@@ -585,20 +597,24 @@
           <t>සුබ දවසක් වේවා හැමෝටම පරිස්සමින් යමන් එහෙනම්.</t>
         </is>
       </c>
-      <c r="E6" s="0" t="n"/>
-      <c r="F6" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>සුබ දවසක් වේවා හැමෝටම පරිස්සමින් යමන් එහෙන්ම්.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Greetings</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "suba dwasak wewa" — a traditional Sinhala blessing phrase commonly used as a formal greeting or farewell.</t>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "suba dwasak wewa"</t>
         </is>
       </c>
     </row>
@@ -615,27 +631,32 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>ayubowan mchn khmda uba?</t>
+          <t>suba udesanak weewa mchn!</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>ආයුබෝවන් මචන් කොහොමද උඹ?</t>
-        </is>
-      </c>
-      <c r="F7" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
+          <t>සුබ උදෑසනක් වේවා මචන්!</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>සුබ උදෑසනක් වීවා මචන්!</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Greetings</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "ayubowan" — the standard Sinhala cultural greeting meaning "may you live long", directly matching the greetings input type.</t>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "suba udesanak weewa"</t>
         </is>
       </c>
     </row>
@@ -660,24 +681,24 @@
           <t>පොඩ්ඩක් බලලා මට කියනවද වෙලා තියෙන දේ ටික?</t>
         </is>
       </c>
-      <c r="E8" s="0" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>පොඩ්ඩක් බලලා මට කියනවද වෙලා තියෙන දේ ට්ක?</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Requests</t>
         </is>
       </c>
-      <c r="F8" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>Rationale: "poddak blala mata kiyanawada" is a polite request asking someone to check and report back, matching the requests input type.</t>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: The user is politely asking someone to check and report back.</t>
         </is>
       </c>
     </row>
@@ -702,19 +723,24 @@
           <t>අනේ පොඩ්ඩක් ඒක දීපන්කෝ බන්.</t>
         </is>
       </c>
-      <c r="F9" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>අනේ පද්දක් එක දීපන්කෝ බන්.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Requests</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "ane pddk eka deepanko" — "ane" and "deepanko" are request softeners in Singlish; the sentence is a polite ask to share something.</t>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "ane pddk eka deepanko"</t>
         </is>
       </c>
     </row>
@@ -726,37 +752,37 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>eka nam sira kathaawa ehemama tama wechche eda.</t>
+          <t>ow bnn ekane mn edama ubata kiwwe oka ohoma wei kyla. uba ahune nane mage kthaawa eda. mama kiwwa neda e welawe wena dewal ekka baluwama mehema wena eka thama godakma hodama de kiyala. dan ithin wela iwarane bnn, ek nisa apita me gana passe welaawaka nidahase katha karamu. mama heta anidda patte ennamko ehenam apita puluwan e welaawata meka gana loku chat ekak danna ehenam theruwan saranai parissamen.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>ඒක නම් සිරා කතාව එහෙමම තමා වෙච්චේ එදා.</t>
-        </is>
-      </c>
-      <c r="E10" s="0" t="inlineStr">
-        <is>
-          <t>රෙපන්ස්</t>
-        </is>
-      </c>
-      <c r="F10" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
+          <t>ඔව් බන් ඒකනේ මං එදාම උඹට කිව්වේ ඕක ඔහොම වෙයි කියලා. උඹ ඇහුවේ නෑනේ මගේ කතාව එදා. මම කිව්වා නේද ඒ වෙලාවේ වෙන දේවල් එක්ක බැලුවම මෙහෙම වෙන එක තමා ගොඩක්ම හොඳම දේ කියලා. දැන් ඉතින් වෙලා ඉවරනේ බන්, ඒක නිසා අපිට මේ ගැන පස්සේ වෙලාවක නිදහසේ කතා කරමු. මම හෙට අනිද්දා පැත්තේ එන්නම්කෝ එහෙනම් අපිට පුළුවන් ඒ වෙලාවට මේක ගැන ලොකු chat එකක් දාන්න එහෙනම් තෙරුවන් සරණයි පරිස්සමෙන්.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ඔව් බන් ඒකනේ මන් එදාම උබට කිව්වේ ඕක ඔහොම වෙයි කියලා. උඹ ඇහුනේ නෑනේ මගේ කතාව එදා. මම කිව්වා නේද ඒ වෙලාවේ වෙන දේවල් එක්ක බැලුවාම මෙහෙම වෙන එක තමා ගොඩක්ම හොදම දේ කියලා. දැන් ඉතින් වෙලා ඉවරනේ බන්, එක් නිසා අපිට මේ ගාන පස්සේ වෙලාවක නිදහසේ කතා කරමු. මම හෙට අනිද්දා පට්ටේ එන්නම්කො එහෙනම් අපිට පුළුවන් ඒ වෙලාවට මේක ගාන ලොකු චාට් එකක් දාන්න එහෙනම් තෙරුවන් සරනයි පරිස්සමෙන්.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Responses</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>Rationale: "eka nam sira kathaawa ehemama tama wechcha" is an affirmative response confirming that something happened exactly as discussed, matching the responses input type.</t>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: The entire 399-character block is an extended affirmative response to a previous event ("ow bnn ekane mn edama ubata kiwwe").</t>
         </is>
       </c>
     </row>
@@ -768,32 +794,37 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>ow ow eka hri mama eda gya.</t>
+          <t>oww oww eeka tma matath hithenne dn karanna deyak na.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>ඔව් ඔව් ඒක හරි මම එදා ගියා.</t>
-        </is>
-      </c>
-      <c r="F11" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
+          <t>ඔව් ඔව් ඒක තමා මටත් හිතෙන්නේ දැන් කරන්න දෙයක් නෑ.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ඔව් ඔව් ඒක තමයි මටත් හිතෙන්නේ දැන් කරන්න දෙයක් නෑ.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Responses</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "ow ow eka hri" — "ow" is the Singlish affirmative particle (yes), and its repetition with "eka hri" confirms agreement, matching the responses input type.</t>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: The phrase "oww oww" confirms agreement.</t>
         </is>
       </c>
     </row>
@@ -818,24 +849,24 @@
           <t>උඹ හෙමින් හෙමින් වරෙන්කෝ හදිස්සි වෙන්නේ නැතුව.</t>
         </is>
       </c>
-      <c r="E12" s="0" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>උඹ හෙමින් හෙමින් වරෙන්කො හදිස්සි වෙන්නෙ නතුව.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Repeated Words</t>
         </is>
       </c>
-      <c r="F12" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>Repeated words</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "hemin hemin" — the word "hemin" (slowly/carefully) is repeated consecutively, a common Singlish emphasis pattern matching the repeated-words input type.</t>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "hemin hemin"</t>
         </is>
       </c>
     </row>
@@ -852,27 +883,32 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>tkak tkak dila blnna.</t>
+          <t>hmin hmin palayan bn.</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>ටිකක් ටිකක් දීලා බලන්න.</t>
-        </is>
-      </c>
-      <c r="F13" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>Repeated words</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "tkak tkak" — "tkak" (a bit) is repeated, a typical Singlish reduplication pattern used for emphasis, matching the repeated-words input type.</t>
+          <t>හෙමින් හෙමින් පලයන් බන්.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>හ්මින් හ්මින් පලයන් බන්.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Repeated Words</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "hmin hmin"</t>
         </is>
       </c>
     </row>
@@ -897,24 +933,24 @@
           <t>එහෙනම්, අපි හෙට සෙට් වෙමු නේද? අනිවා!! ගින්දර..</t>
         </is>
       </c>
-      <c r="E14" s="0" t="inlineStr">
-        <is>
-          <t>ඉන්පුට්ස් with Punctuation Marks</t>
-        </is>
-      </c>
-      <c r="F14" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with punctuation marks</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>Rationale: The input uses a comma, question mark, and double exclamation ("neda?", "aniwa!!") in one sentence — multiple punctuation types within a single conversational Singlish input.</t>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>එහෙනම්, අපි හෙට set වෙමු නේද? අනිවා!! gndos..</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Punctuation Marks</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: The input uses commas, question marks, and multiple exclamation points.</t>
         </is>
       </c>
     </row>
@@ -939,19 +975,24 @@
           <t>මොකක්ද බන් ඒ?! කියපන්කෝ...</t>
         </is>
       </c>
-      <c r="F15" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with punctuation marks</t>
-        </is>
-      </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "?!" and "..." — the input contains mixed consecutive punctuation (interrobang-style "?!" and ellipsis "..."), testing how the translator handles non-standard punctuation sequences.</t>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>මොකද බන් ඒ?! කියපන්කෝ...</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Punctuation Marks</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: The input features consecutive punctuation marks like '?!' and '...' .</t>
         </is>
       </c>
     </row>
@@ -976,20 +1017,24 @@
           <t>මං නම් කියන්නේ ඔය වැඩේ කරන්න එපා කියලා එයාට.</t>
         </is>
       </c>
-      <c r="E16" s="0" t="n"/>
-      <c r="F16" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>Romanization / Spelling variants</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
-        <is>
-          <t>Rationale: "wedee" uses an extra vowel (double-e) as a non-standard spelling variant of "wede", representing a phonetic spelling deviation from standard Singlish romanization.</t>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>මන් නම් කියන්නේ ඔය වැඩේ කරන්න එපා කියලා එයාට.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Romanization / Spelling Variants</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: The word 'wedee' is written with a double 'e' and 'kranna' omits the 'a'.</t>
         </is>
       </c>
     </row>
@@ -1014,19 +1059,24 @@
           <t>මගේ පොත දීලා යන්න එන්න.</t>
         </is>
       </c>
-      <c r="F17" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>Romanization / Spelling variants</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
-        <is>
-          <t>Rationale: "ptha", "ynn", "enna" are heavily abbreviated variants of "putha", "yanna", "enna" — dropping vowels mid-word is a common informal Singlish romanization pattern.</t>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>මගේ පෘත දීලා යන්න එන්න.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Romanization / Spelling Variants</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: Words are heavily abbreviated by dropping vowels (e.g., 'mge', 'ptha', 'ynn').</t>
         </is>
       </c>
     </row>
@@ -1038,33 +1088,37 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>mage phone eka kadila wena ekak ganna one den.</t>
+          <t>mage laptop eke awlak.</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>මගේ phone එක කැඩිලා වෙන එකක් ගන්න ඕනේ දැන්.</t>
-        </is>
-      </c>
-      <c r="E18" s="0" t="n"/>
-      <c r="F18" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>Isolated English word insertions in Singlish</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "phone" — a single English noun is inserted into an otherwise Singlish sentence ("mage phone eka"), representing the isolated-English-word insertion input type.</t>
+          <t>මගේ laptop එකේ අවුලක්.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>මගේ laptop එකේ අව්ලක්.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Isolated English Word Insertions in Singlish</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: The English word "laptop" is inserted.</t>
         </is>
       </c>
     </row>
@@ -1089,19 +1143,24 @@
           <t>හෙට ලොකු meeting එකක් තියෙනවා.</t>
         </is>
       </c>
-      <c r="F19" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>Isolated English word insertions in Singlish</t>
-        </is>
-      </c>
-      <c r="H19" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "meeting" — a single English noun is embedded in a Singlish sentence ("loku meeting ekak tynwa"), representing an isolated English word insertion.</t>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>හ්ට ලොකු meeting එකක් තියෙනවා.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Isolated English Word Insertions in Singlish</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: The single English word "meeting" is inserted.</t>
         </is>
       </c>
     </row>
@@ -1113,37 +1172,37 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>api end of the day kohomahari project eka demu.</t>
+          <t>machan ara project eka gana baluwama eka nam out of the box hithala karanna one loku wedak thama. mokada apita normal widihata eka complete karanna baha kiyala mata hodatama therenawa dan. eka nisa api end of the day kohoma hari hamoma ekathu wela meka iwara karamu neda. nethnam boss apita loku case ekak dai kiyala mata sure. eka nisa please make sure to complete everything on time machan aniwa.</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>අපි end of the day කොහොමහරි project එක දෙමු.</t>
-        </is>
-      </c>
-      <c r="E20" s="0" t="inlineStr">
+          <t>මචන් අර project එක ගැන බැලුවම ඒක නම් out of the box හිතලා කරන්න ඕනේ ලොකු වැඩක් තමා. මොකද අපිට normal විදිහට ඒක complete කරන්න බැහැ කියලා මට හොඳටම තේරෙනවා දැන්. ඒක නිසා අපි end of the day කොහොම හරි හැමෝම එකතු වෙලා මේක ඉවර කරමු නේද. නැත්නම් boss අපිට ලොකු case එකක් දෙනවා කියලා මට sure. ඒක නිසා please make sure to complete everything on time මචන් අනිවා.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>මචං අර project එක ගැන බැලුවාම ඒක නම් out of the box හිතලා කරන්න ඕනේ ලොකු වැඩක් තමා. මොකද අපිට normal විදිහට එක complete කරන්න බෑ කියලා මට හොදටම තේරෙනවා දැන්. ඒක නිසා අපි end of the day කොහොම හරි හැමෝම එකතු වෙලා මේක ඉවර කරමු නේද. නැත්නම් boss අපිට ලොකු case එකක් දායි කියලා මට sure. ඒක නිසා please make sure to complete everything on time මචන් අනිවා.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>Multi-Word English Phrases in Singlish</t>
         </is>
       </c>
-      <c r="F20" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>Multi-word English phrases in Singlish</t>
-        </is>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "end of the day" — a complete multi-word English idiomatic phrase is used inline within a Singlish sentence, matching the multi-word English phrase input type.</t>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: The phrases "out of the box", "end of the day", and "make sure to complete everything on time" are used.</t>
         </is>
       </c>
     </row>
@@ -1168,19 +1227,24 @@
           <t>ඒක නම් out of the box හිතලා කරපු වැඩක් තමා.</t>
         </is>
       </c>
-      <c r="F21" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>Multi-word English phrases in Singlish</t>
-        </is>
-      </c>
-      <c r="H21" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "out of the box" — a complete multi-word English idiomatic expression is embedded in a Singlish sentence, matching the multi-word English phrase input type.</t>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ඒක නම් out of the box හිතලා කරපු වැඩක් තමයි.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Multi-Word English Phrases in Singlish</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: The phrase "out of the box" is used.</t>
         </is>
       </c>
     </row>
@@ -1197,32 +1261,32 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>oya server eka down wela pen eke dapan files tka.</t>
+          <t>ane mge wifi routereka rstart kralat hri giye na bn.</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>ඔය server එක down වෙලා pen එකේ දාපන් files ටික.</t>
-        </is>
-      </c>
-      <c r="E22" s="0" t="inlineStr">
+          <t>අනේ මගේ wifi router එක restart කරලත් හරි ගියේ නෑ බන්.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>අනේ මගේ wifi router එක start කරලාත් හරි ගියේ නෑ බන්.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>English Digital Terms in Singlish</t>
         </is>
       </c>
-      <c r="F22" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>English digital terms in Singlish</t>
-        </is>
-      </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "server", "down", "fix" — three English digital/technical terms are embedded within a conversational Singlish sentence, matching the English digital terms input type.</t>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: The digital terms ""wifi"", ""router"", and ""restart"" are used.</t>
         </is>
       </c>
     </row>
@@ -1247,19 +1311,24 @@
           <t>wifi password එක මොකක්ද?</t>
         </is>
       </c>
-      <c r="F23" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>English digital terms in Singlish</t>
-        </is>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "wifi", "password" — two common English digital terms are used in a Singlish question, matching the English digital terms input type.</t>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>wifi password එක මොකද?</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>English Digital Terms in Singlish</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: The digital terms "wifi" and "password" are present.</t>
         </is>
       </c>
     </row>
@@ -1284,24 +1353,24 @@
           <t>උඹ telegram එකෙන් එවන්න ඒක ලේසි whatsapp වලට.</t>
         </is>
       </c>
-      <c r="E24" s="0" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>උඹ ටෙලිග්රම් එකෙන් එවන්න එක ලේසි වට්සප්ප් වලට.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>Platform/App Names in Singlish</t>
         </is>
       </c>
-      <c r="F24" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>Platform / app names in Singlish</t>
-        </is>
-      </c>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "telegram", "watsapp" — two social media / messaging platform names are referenced inline in a Singlish sentence, matching the platform/app names input type.</t>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "telegram" and "watsapp"</t>
         </is>
       </c>
     </row>
@@ -1326,19 +1395,24 @@
           <t>instagram post එක දාන්න.</t>
         </is>
       </c>
-      <c r="F25" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="inlineStr">
-        <is>
-          <t>Platform / app names in Singlish</t>
-        </is>
-      </c>
-      <c r="H25" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "instagram" — the name of a major social media platform is used directly in a Singlish command, matching the platform/app names input type.</t>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Instagram post එක දාන්න.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Platform/App Names in Singlish</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "instagram"</t>
         </is>
       </c>
     </row>
@@ -1363,24 +1437,24 @@
           <t>මම CV එක එවන්නම් පුළුවන් තරම් ASAP බලන්න.</t>
         </is>
       </c>
-      <c r="E26" s="0" t="inlineStr">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>මම CV ඒක එවන්නම් පුළුවන් තරම් ASAP බලන්න.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>English Abbreviations/Acronyms in Singlish</t>
         </is>
       </c>
-      <c r="F26" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="inlineStr">
-        <is>
-          <t>English abbreviations / acronyms in Singlish</t>
-        </is>
-      </c>
-      <c r="H26" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "CV" (curriculum vitae) and "ASAP" (as soon as possible) — two English acronyms are used in a single Singlish sentence, matching the abbreviations/acronyms input type.</t>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "CV" and "ASAP"</t>
         </is>
       </c>
     </row>
@@ -1405,19 +1479,24 @@
           <t>මට ETA එක කියන්න පුළුවන්ද?</t>
         </is>
       </c>
-      <c r="F27" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>English abbreviations / acronyms in Singlish</t>
-        </is>
-      </c>
-      <c r="H27" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "ETA" (estimated time of arrival) — an English acronym is inserted in a Singlish question, matching the abbreviations/acronyms input type.</t>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>මට ETA ඒක කියන්න පුළුවන්ද?</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>English Abbreviations/Acronyms in Singlish</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "ETA"</t>
         </is>
       </c>
     </row>
@@ -1442,20 +1521,24 @@
           <t>හෙට මීට වඩා ටිකක් ලොකු lab එකකට යන්න වෙනවා.</t>
         </is>
       </c>
-      <c r="E28" s="0" t="n"/>
-      <c r="F28" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G28" s="7" t="inlineStr">
-        <is>
-          <t>English clipped forms in Singlish</t>
-        </is>
-      </c>
-      <c r="H28" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "lab" — a clipped form of "laboratory" is used in a Singlish sentence, matching the English clipped forms input type.</t>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>හෙට මිට වඩා ටිකක් ලොකු lab එකකට යන්න වෙනවා.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>English Clipped Forms in Singlish</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "lab" is used instead of laboratory.</t>
         </is>
       </c>
     </row>
@@ -1480,19 +1563,24 @@
           <t>exam එකක් තියෙනවා හෙට උදේම.</t>
         </is>
       </c>
-      <c r="F29" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
-        <is>
-          <t>English clipped forms in Singlish</t>
-        </is>
-      </c>
-      <c r="H29" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "exam" — a clipped form of "examination" is embedded in a Singlish sentence, matching the English clipped forms input type.</t>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>exam එකක් තියෙනවා හ්ට උදේම.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>English Clipped Forms in Singlish</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "exam" is used instead of examination.</t>
         </is>
       </c>
     </row>
@@ -1517,20 +1605,24 @@
           <t>හෙට නුගේගොඩ junction එක ගාව මං ඉන්නම් වේලාසන.</t>
         </is>
       </c>
-      <c r="E30" s="0" t="n"/>
-      <c r="F30" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
-        <is>
-          <t>Place names embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H30" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "nugegoda junction" — the Sri Lankan place name "Nugegoda" is directly embedded in a Singlish sentence to describe a meeting location, matching the place names input type.</t>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>හෙට නුගේගොඩ junction එක ගාව මන් ඉන්නම් වේල්සන.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Place Names Embedded in Singlish</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: The location "nugegoda" is explicitly mentioned.</t>
         </is>
       </c>
     </row>
@@ -1555,19 +1647,24 @@
           <t>mt lavinia පැත්තේ යමු අද.</t>
         </is>
       </c>
-      <c r="F31" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
-        <is>
-          <t>Place names embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H31" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "mt lavinia" — the Sri Lankan coastal locality "Mt. Lavinia" is embedded in a Singlish suggestion, matching the place names input type.</t>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>මට ලවිනියා පැත්තේ යමු අද.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>Place Names Embedded in Singlish</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: The location "mt lavinia" is explicitly mentioned.</t>
         </is>
       </c>
     </row>
@@ -1579,33 +1676,37 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>e wede chamara aiyata deela tyenne baya wenna epa.</t>
+          <t>mama eda thathsarata kiwwa me dawas wala poddak busy nisa passe welawaka wede karala dennam kiyala. eth eya mata aith call karala ahanawa kawadda eka iwara karala denna puluwan wenne kiyala. mama nimal ayyath ekkath poddak katha karala baluwa eya kiyanawath me dawas wala loku weda thogayak thiyenawa kiyala. eka nisa apita sathi dekak wath yai meka iwara karala thathsarata denna puluwan wenakota.</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>ඒ වැඩේ චාමර අයියට දීලා තියෙන්නේ බය වෙන්න එපා.</t>
-        </is>
-      </c>
-      <c r="E32" s="0" t="n"/>
-      <c r="F32" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G32" s="7" t="inlineStr">
-        <is>
-          <t>Person names embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H32" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "chamara aiya" — the person name "Chamara" with the kinship title "aiya" (elder brother) is embedded in a Singlish sentence, matching the person names input type.</t>
+          <t>මම එදා තත්සරට කිව්වා මේ දවස් වල පොඩ්ඩක් busy නිසා පස්සේ වෙලාවක වැඩේ කරලා දෙන්නම් කියලා. ඒත් එයා මට ආයෙත් call කරලා අහනවා කවද්ද ඒක ඉවර කරලා දෙන්න පුළුවන් වෙන්නේ කියලා. මම නිමල් අයියත් එක්කත් පොඩ්ඩක් කතා කරලා බැලුවා එයා කියනවාත් මේ දවස් වල ලොකු වැඩ තොගයක් තියෙනවා කියලා. ඒක නිසා අපිට සති දෙකක් වත් යයි මේක ඉවර කරලා තත්සරට දෙන්න පුළුවන් වෙනකොට.</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>මම එදා තත්සරට කිව්වා මේ දවස් වල පොඩ්ඩක් busy නිසා පස්සේ වෙලාවක වැඩේ කරලා දෙන්නම් කියලා. ඒත් එයා මට ආයේ call කරලා අහනවා කවද්ද ඒක ඉවර කරලා දෙන්න පුළුවන් වෙන්නේ කියලා. මම නිමල් අය්යත් එක්කත් පොඩ්ඩක් කතා කරලා බැලුවා එයා කියනවත් මේ දවස් වල ලොකු වැඩ තොගයක් තියෙනවා කියලා. ඒක නිසා අපිට සති දෙකක් වත් යයි මේක ඉවර කරලා තත්සරට දෙන්න පුළුවන් වෙනකොට.</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Person Names Embedded in Singlish</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: The person names "thathsarata" (Thathsara) and "nimal" are embedded within the 400-character text.</t>
         </is>
       </c>
     </row>
@@ -1617,32 +1718,37 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>nimal mchn mokda krnne?</t>
+          <t>sachinthaya ta kiala e wede welsnama goda damu neda.</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>නිමල් මචන් මොකද කරන්නේ?</t>
-        </is>
-      </c>
-      <c r="F33" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G33" s="7" t="inlineStr">
-        <is>
-          <t>Person names embedded in Singlish</t>
-        </is>
-      </c>
-      <c r="H33" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "nimal" — the person name "Nimal" is used as the subject of a Singlish question, matching the person names input type.</t>
+          <t>සචින්තයට කියලා ඒ වැඩේ වේලාසනම ගොඩ දාමු නේද.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>සචින්තය ට කියලා ඒ වැඩේ වේල්ස්නාම ගොඩ දාමු නේද.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>Person Names Embedded in Singlish</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: The person name "sachinthaya" (Sachintha) is used.</t>
         </is>
       </c>
     </row>
@@ -1667,20 +1773,24 @@
           <t>මට 10ක් වත් එවනවද අර සල්ලි වලින් අඩු කරලා.</t>
         </is>
       </c>
-      <c r="E34" s="0" t="n"/>
-      <c r="F34" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with numbers and numeric suffixes</t>
-        </is>
-      </c>
-      <c r="H34" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "10k" — the numeral "10" is combined with the Singlish/English suffix "k" (thousand), forming a mixed numeric token, matching the numbers and numeric suffixes input type.</t>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>මට 10ක් වත් එවනවද අර සල්ලි වෙලින් අඩු කරලා.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Numbers and Numeric Suffixes</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "10k" combines a number with a Singlish suffix.</t>
         </is>
       </c>
     </row>
@@ -1705,19 +1815,24 @@
           <t>උඹ 3වෙනි පේළියේ ඉන්න.</t>
         </is>
       </c>
-      <c r="F35" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with numbers and numeric suffixes</t>
-        </is>
-      </c>
-      <c r="H35" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "3weni" — the numeral "3" is combined with the Sinhala ordinal suffix "weni" (third), forming a numeric–suffix token, matching the numbers and numeric suffixes input type.</t>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>උඹ 3වෙනි පේලියේ ඉන්න.</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Numbers and Numeric Suffixes</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "3weni" combines a number with a Singlish suffix.</t>
         </is>
       </c>
     </row>
@@ -1742,20 +1857,24 @@
           <t>අර රු 5000 දීපන්කෝ අද හවසට ආපහු දෙන්නම්.</t>
         </is>
       </c>
-      <c r="E36" s="0" t="n"/>
-      <c r="F36" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with currency</t>
-        </is>
-      </c>
-      <c r="H36" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "rs 5000" — the Sri Lankan currency abbreviation "rs" (rupees) is used with a numeral amount in a Singlish sentence, matching the currency input type.</t>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>අර රුස් 5000 දීපංකෝ අද හවසට ආපහු දෙන්නම්.</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Currency</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "rs 5000"</t>
         </is>
       </c>
     </row>
@@ -1772,27 +1891,32 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>$50 kiyanne keeyada dan?</t>
+          <t>usd 10k kiynne keeyda?</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>$50 කියන්නේ කීයද දැන්?</t>
-        </is>
-      </c>
-      <c r="F37" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with currency</t>
-        </is>
-      </c>
-      <c r="H37" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "$50" — the US dollar symbol "$" is used with a numeral in a Singlish question, matching the currency input type.</t>
+          <t>USD 10ක් කියන්නේ කීයද?</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>උස්ඩ් 10ක් කියන්නේ කීයද?</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Currency</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "usd 10k"</t>
         </is>
       </c>
     </row>
@@ -1817,20 +1941,24 @@
           <t>අපිට හෙට 10.30am වෙද්දී office ඉන්න පුළුවන්ද කියලා දාපන්.</t>
         </is>
       </c>
-      <c r="E38" s="0" t="n"/>
-      <c r="F38" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G38" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with time formats</t>
-        </is>
-      </c>
-      <c r="H38" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "10.30am" — a 12-hour clock time with AM/PM suffix is embedded in a Singlish sentence, matching the time formats input type.</t>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>අපිට හෙට 10.30am වෙද්දි office ඉන්න පුළුවන්ද කියලා දාපන්.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Time Formats</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "10.30am"</t>
         </is>
       </c>
     </row>
@@ -1855,19 +1983,24 @@
           <t>හවස් 5pm වෙනකොට මං එන්නම්.</t>
         </is>
       </c>
-      <c r="F39" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with time formats</t>
-        </is>
-      </c>
-      <c r="H39" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "5pm" — a 12-hour clock time with a PM suffix is used in a Singlish statement, matching the time formats input type.</t>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>හවස 5pm වෙනකොට මන් එන්නම්.</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Time Formats</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "5pm"</t>
         </is>
       </c>
     </row>
@@ -1892,20 +2025,24 @@
           <t>මගේ birthday එක තියෙන්නේ 2026-10-15 මතක තියා ගනින්.</t>
         </is>
       </c>
-      <c r="E40" s="0" t="n"/>
-      <c r="F40" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G40" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with dates</t>
-        </is>
-      </c>
-      <c r="H40" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "2026-10-15" — an ISO 8601 formatted date (YYYY-MM-DD) is embedded in a Singlish sentence, matching the dates input type.</t>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>මගේ birthday එක තියෙන්නේ 2026-10-15 මාතෘකා තියා ගනින්.</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Dates</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "2026-10-15"</t>
         </is>
       </c>
     </row>
@@ -1930,19 +2067,24 @@
           <t>oct 15 තමා වැඩේ ඉවර.</t>
         </is>
       </c>
-      <c r="F41" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with dates</t>
-        </is>
-      </c>
-      <c r="H41" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "oct 15" — an abbreviated month name followed by a day number is used in a Singlish sentence, matching the dates input type.</t>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>oct 15 තාම වැඩේ ඉවර.</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Dates</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "oct 15"</t>
         </is>
       </c>
     </row>
@@ -1967,20 +2109,24 @@
           <t>ගෙදර ඉඳලා town එකට 5km තියෙනවා පයින් යමු අපි.</t>
         </is>
       </c>
-      <c r="E42" s="0" t="n"/>
-      <c r="F42" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G42" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with units of measurement</t>
-        </is>
-      </c>
-      <c r="H42" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "5km" — the metric distance unit "km" (kilometres) is combined with a numeral in a Singlish sentence, matching the units of measurement input type.</t>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ගෙදර ඉදලා town එකට 5km තියෙනවා පයින් යමු අපි.</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Unit of Measurements</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "5km"</t>
         </is>
       </c>
     </row>
@@ -2005,19 +2151,24 @@
           <t>පිටි 2kg ගෙන්න ඇතුව.</t>
         </is>
       </c>
-      <c r="F43" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G43" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with units of measurement</t>
-        </is>
-      </c>
-      <c r="H43" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "2kg" — the metric weight unit "kg" (kilograms) is combined with a numeral in a Singlish command, matching the units of measurement input type.</t>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>පිටි 2kg ගේන්න ආට්ව.</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Unit of Measurements</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: "2kg"</t>
         </is>
       </c>
     </row>
@@ -2042,20 +2193,24 @@
           <t>සුපිරි බන් උඹ නම් පට්ට ඩයල් එකක් නේ සිරාවටම.</t>
         </is>
       </c>
-      <c r="E44" s="0" t="n"/>
-      <c r="F44" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with slang and casual phrasing</t>
-        </is>
-      </c>
-      <c r="H44" s="8" t="inlineStr">
-        <is>
-          <t>Rationale: Uses heavy Singlish slang — "patta dial" (awesome call/move), "sirawatama" (absolutely perfectly), "bn" (bana/friend) — all informal colloquial tokens matching the slang and casual phrasing input type.</t>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>සුපිරි බන් උඹ නම් පට්ට dial එකක් නෑ සිරාවටම.</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Slang and Casual Phrasing</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: Uses heavy colloquial slang like "patta dial" and "sirawatama".</t>
         </is>
       </c>
     </row>
@@ -2067,32 +2222,37 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>uuta mala panala tyenne.</t>
+          <t>uuba nam maha patta gembek bnn kiyala thama mata kiyanna wenne. mokada uba eda e katha karapu widiha nam mata echchara alluwe naha machan. eka nisa thama mama ubata katha nokara hitiye me tike. anika uba patta dial ekak kiyala hithagena hitigata ehema baha ne ban samaje ekka inna kota. sirawatama kiyanawanm mata uba ekka me gana ayeth katha karanna hithenneth naha ban mokada uba echcharatama epa wela.</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>ඌට මල පැනලා තියෙන්නේ.</t>
-        </is>
-      </c>
-      <c r="F45" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G45" s="7" t="inlineStr">
-        <is>
-          <t>Inputs with slang and casual phrasing</t>
-        </is>
-      </c>
-      <c r="H45" s="8" t="inlineStr">
-        <is>
-          <t>Rationale: "mala panala" is an idiomatic Singlish slang phrase meaning something went very wrong/crazy; it is an informal colloquial expression matching the slang and casual phrasing input type.</t>
+          <t>උඹ නම් මහා පට්ට ගෙම්බෙක් බන් කියලා තමා මට කියන්න වෙන්නේ. මොකද උඹ එදා ඒ කතා කරපු විදිහ නම් මට එච්චර ඇල්ලුවේ නැහැ මචන්. ඒක නිසා තමා මම උඹට කතා නොකර හිටියේ මේ ටිකේ. අනික උඹ පට්ට ඩයල් එකක් කියලා හිතාගෙන හිටියට එහෙම බැහැ නේ බන් සමාජේ එක්ක ඉන්න කොට. සිරාවටම කියනවා නම් මට උඹ එක්ක මේ ගැන ආයෙත් කතා කරන්න හිතෙන්නෙත් නැහැ බන් මොකද උඹ එච්චරටම එපා වෙලා.</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>උඋබ නම් මහ පට්ට ගෙම්බෙක් බන් කියලා තමා මට කියන්න වෙන්නේ. මොකද උඹ එදා ඒ කතා කරපු විදිහ නම් මට එච්චර අල්ලුවෙ නැහැ මචං. ඒක නිසා තමා මම උබට කතා නොකර හිටියේ මේ ටිකේ. අනික උඹ පට්ට dial එකක් කියල හිතාගෙන හිටිගට එහෙම බහ නෑ බං සමාජෙ එක්ක ඉන්න කොට. සිරාවටම කියනවන්ම් මට උඹ එක්ක මේ ගාන ආයෙත් කතා කරන්න හිතෙන්නෙත් නැහැ බං මොකද උඹ එච්චරටම එපා වෙලා.</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>Inputs with Slang and Casual Phrasing</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: The long 405-character text relies heavily on extreme colloquial slang like "patta gembek" and "patta dial ekak".</t>
         </is>
       </c>
     </row>
@@ -2109,28 +2269,32 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>oya wede gena igena ganna www.w3schools.com yman.</t>
+          <t>mage web eka https://aluth.lk eken ghin balanna puluwan.</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>ඔය වැඩේ ගැන ඉගෙන ගන්න www.w3schools.com යමන්.</t>
-        </is>
-      </c>
-      <c r="E46" s="0" t="n"/>
-      <c r="F46" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G46" s="7" t="inlineStr">
-        <is>
-          <t>Online identifiers in Singlish</t>
-        </is>
-      </c>
-      <c r="H46" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "www.w3schools.com" — a full URL is embedded mid-sentence in a Singlish statement, matching the online identifiers input type.</t>
+          <t>මගේ web එක https://aluth.lk එකෙන් ගිහින් බලන්න පුළුවන්.</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>මගේ වෙබ් එක https://aluth.lk ඒකෙන් ගිහින් බලන්න පුළුවන්.</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>Online Indentifiers in Singlish</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: Contains the URL "https://aluth.lk"</t>
         </is>
       </c>
     </row>
@@ -2155,19 +2319,24 @@
           <t>@nimal123 tag කරලා දාපන්.</t>
         </is>
       </c>
-      <c r="F47" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr">
-        <is>
-          <t>Online identifiers in Singlish</t>
-        </is>
-      </c>
-      <c r="H47" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "@nimal123" — a social media handle (@ + username) is used in a Singlish command, matching the online identifiers input type.</t>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>@නිමල්123 tag කරලා දාපන්.</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>Online Indentifiers in Singlish</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: Contains the handle "@nimal123"</t>
         </is>
       </c>
     </row>
@@ -2184,28 +2353,32 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>eka ahala mata hina gihin pana giya 😂 mara seen eka.</t>
+          <t>ammo eka dakkama mawa pichchuna 🥵🔥 sraa kathawa.</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>ඒක අහලා මට හිනා ගිහින් පණ ගියා 😂 මාර සීන් එක.</t>
-        </is>
-      </c>
-      <c r="E48" s="0" t="n"/>
-      <c r="F48" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="inlineStr">
-        <is>
-          <t>Inputs containing emojis</t>
-        </is>
-      </c>
-      <c r="H48" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: 😂 — the "face with tears of joy" emoji is embedded mid-sentence within a Singlish statement, matching the emojis input type.</t>
+          <t>අම්මෝ ඒක දැක්කම මාව පිච්චුනා 🥵🔥 සිරා කතාව.</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>අම්මෝ ඒක දැක්කම මාව පිච්චුණා 🥵🔥 ශ්‍ර කථාව.</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>Inputs Containing Emojis</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: Contains the 🥵 and 🔥 emojis.</t>
         </is>
       </c>
     </row>
@@ -2230,19 +2403,24 @@
           <t>congratzz මචන් 🎉💪 එළ.</t>
         </is>
       </c>
-      <c r="F49" s="0" t="inlineStr">
-        <is>
-          <t>UI Error</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="inlineStr">
-        <is>
-          <t>Inputs containing emojis</t>
-        </is>
-      </c>
-      <c r="H49" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: 🎉💪 — a "party popper" and "flexed bicep" emoji are used together in a short Singlish congratulatory message, matching the emojis input type.</t>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>congratzz මචන් 🎉💪 එල.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Inputs Containing Emojis</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>Evidence: Contains the 🎉 and 💪 emojis.</t>
         </is>
       </c>
     </row>
@@ -2267,20 +2445,24 @@
           <t>frontend එක build කරද්දි error එකක් ආවා පොඩ්ඩක් බලන්න.</t>
         </is>
       </c>
-      <c r="E50" s="0" t="n"/>
-      <c r="F50" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr">
-        <is>
-          <t>English digital terms in Singlish</t>
-        </is>
-      </c>
-      <c r="H50" s="8" t="inlineStr">
-        <is>
-          <t>Evidence: "frontend", "build", "error" — three technical software development terms are embedded in a conversational Singlish sentence, matching the English digital terms input type.</t>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ෆ්රොන්ට්එන්ඩ් එක බිල්ඩ් කරද්දී error එකක් ආවා පොඩ්ඩක් බලන්න.</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>Isolated English Word Insertions in Singlish</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: Testing technical developer jargon mixed into conversational text.</t>
         </is>
       </c>
     </row>
@@ -2305,20 +2487,24 @@
           <t>හැමෝම එකතු වෙලා මේ වැඩේ ලේසියෙන් ගොඩ දාගමු කොල්ලෝ.</t>
         </is>
       </c>
-      <c r="E51" s="0" t="n"/>
-      <c r="F51" s="0" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
-        <is>
-          <t>Romanization / Spelling variants</t>
-        </is>
-      </c>
-      <c r="H51" s="8" t="inlineStr">
-        <is>
-          <t>Rationale: "hmoma" (for "hamoma"), "wdee" (for "wede"), "dgamu" (for "dagamu") — extreme vowel-dropping abbreviations typical of fast Singlish group-chat typing, matching the romanization/spelling variants input type.</t>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>හැමෝම එකතු වෙලා මී වැඩී ලේසියෙන් ගොඩ දාගමු කොල්ලෝ.</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>Romanization / Spelling Variants</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>Rationale: Testing extreme abbreviation ('hmoma', 'wdee', 'dgamu') commonly found in group chats.</t>
         </is>
       </c>
     </row>

</xml_diff>